<commit_message>
Sync JobStreet batch candidates into master recruiting DB
</commit_message>
<xml_diff>
--- a/projects/recruiting-id/SeahubMedia_ID_Recruiting_CandidateDB_CN.xlsx
+++ b/projects/recruiting-id/SeahubMedia_ID_Recruiting_CandidateDB_CN.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC1"/>
+  <dimension ref="A1:AC21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -609,6 +609,646 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Rafael Gary</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>+6281285929651</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>+6281285929651</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>https://id.employer.seek.com/id/candidates/?jobid=89488639&amp;selected=2013697082&amp;s=Shortlist</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>imported 2026-02-19T09:41:36 from JobStreet_Candidates_Batch1_20.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Susan Cu</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>+6281285887748</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>+6281285887748</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>https://id.employer.seek.com/id/candidates/?jobid=89488639&amp;selected=2013540695</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>imported 2026-02-19T09:41:36 from JobStreet_Candidates_Batch1_20.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Puspita Nabila Martha</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>+628889218494</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>+628889218494</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>https://id.employer.seek.com/id/candidates/?jobid=89488639&amp;selected=2013528360&amp;s=Shortlist</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>imported 2026-02-19T09:41:36 from JobStreet_Candidates_Batch1_20.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Moh Ainul Yakin</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>+6281284587940</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>+6281284587940</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>https://id.employer.seek.com/id/candidates/?jobid=89488639&amp;selected=2013436180</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>imported 2026-02-19T09:41:36 from JobStreet_Candidates_Batch1_20.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Dwi Safitri</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>+6281995588001</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>+6281995588001</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>https://id.employer.seek.com/id/candidates/?jobid=89488639&amp;selected=2012789873</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>imported 2026-02-19T09:41:36 from JobStreet_Candidates_Batch1_20.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Ari Apriliyani</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>+6283894954955</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>+6283894954955</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>https://id.employer.seek.com/id/candidates/?jobid=89488639&amp;selected=2012451154</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>imported 2026-02-19T09:41:36 from JobStreet_Candidates_Batch1_20.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Aulia Amalia Ashari</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>+6287817095821</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>+6287817095821</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>https://id.employer.seek.com/id/candidates/?jobid=89488639&amp;selected=2012379843&amp;s=Rejected</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>imported 2026-02-19T09:41:36 from JobStreet_Candidates_Batch1_20.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Manuarang Sinambela</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>+6281386010216</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>+6281386010216</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>https://id.employer.seek.com/id/candidates/?jobid=89488639&amp;selected=2012334133&amp;s=Rejected</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>imported 2026-02-19T09:41:36 from JobStreet_Candidates_Batch1_20.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>inrianto .</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>+62085881765868</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>+62085881765868</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>https://id.employer.seek.com/id/candidates/?jobid=89488639&amp;selected=2012262711</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>imported 2026-02-19T09:41:36 from JobStreet_Candidates_Batch1_20.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Arlita Alistia</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>+6289611550024</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>+6289611550024</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>https://id.employer.seek.com/id/candidates/?jobid=89488639&amp;selected=2012200128&amp;s=Shortlist</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>imported 2026-02-19T09:41:36 from JobStreet_Candidates_Batch1_20.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Refitha Rachmadanisya</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>+6285732238300</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>+6285732238300</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>https://id.employer.seek.com/id/candidates/?jobid=89488639&amp;selected=2012165468&amp;s=Rejected</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>imported 2026-02-19T09:41:36 from JobStreet_Candidates_Batch1_20.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Annisa Fitri Salsabila</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>+6285121119295</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>+6285121119295</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>https://id.employer.seek.com/id/candidates/?jobid=89488639&amp;selected=2012165244</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>imported 2026-02-19T09:41:36 from JobStreet_Candidates_Batch1_20.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Fransiska Rikha Krismasdayanti</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>+6289603404224</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>+6289603404224</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>https://id.employer.seek.com/id/candidates/?jobid=89488639&amp;selected=2012126169</t>
+        </is>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>imported 2026-02-19T09:41:36 from JobStreet_Candidates_Batch1_20.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Deviana Putri Yunisa</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>+6287845985397</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>+6287845985397</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>https://id.employer.seek.com/id/candidates/?jobid=89488639&amp;selected=2012109216&amp;s=Rejected</t>
+        </is>
+      </c>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>imported 2026-02-19T09:41:36 from JobStreet_Candidates_Batch1_20.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Yolanda Dewi Ariyanti</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>+6282123505473</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>+6282123505473</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>https://id.employer.seek.com/id/candidates/?jobid=89488639&amp;selected=2012090971&amp;s=Rejected</t>
+        </is>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>imported 2026-02-19T09:41:36 from JobStreet_Candidates_Batch1_20.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Mochamad Ulul Azmi Wira Utama</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>+6281285802247</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>+6281285802247</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>https://id.employer.seek.com/id/candidates/?jobid=89488639&amp;selected=2012086796</t>
+        </is>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>imported 2026-02-19T09:41:36 from JobStreet_Candidates_Batch1_20.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Fajar Adhi</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>+6281328262527</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>+6281328262527</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>https://id.employer.seek.com/id/candidates/?jobid=89488639&amp;selected=2012069874</t>
+        </is>
+      </c>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>imported 2026-02-19T09:41:36 from JobStreet_Candidates_Batch1_20.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Regina Sugito</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>+628112630086</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>+628112630086</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>https://id.employer.seek.com/id/candidates/?jobid=89488639&amp;selected=2012059494</t>
+        </is>
+      </c>
+      <c r="AC19" t="inlineStr">
+        <is>
+          <t>imported 2026-02-19T09:41:36 from JobStreet_Candidates_Batch1_20.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Yosua Ferdyanto</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>+6281293976473</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>+6281293976473</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>https://id.employer.seek.com/id/candidates/?jobid=89488639&amp;selected=2012057626&amp;s=Shortlist</t>
+        </is>
+      </c>
+      <c r="AC20" t="inlineStr">
+        <is>
+          <t>imported 2026-02-19T09:41:36 from JobStreet_Candidates_Batch1_20.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Nathan Adriano Wibowo</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>+6281211058757</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>+6281211058757</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>https://id.employer.seek.com/id/candidates/?jobid=89488639&amp;selected=2012015073</t>
+        </is>
+      </c>
+      <c r="AC21" t="inlineStr">
+        <is>
+          <t>imported 2026-02-19T09:41:36 from JobStreet_Candidates_Batch1_20.xlsx</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:AC1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>